<commit_message>
penambahan fitur pengunjung dan laporan pengunjung
</commit_message>
<xml_diff>
--- a/public/template/template_import_buku.xlsx
+++ b/public/template/template_import_buku.xlsx
@@ -1,26 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24729"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\felix\Downloads\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A8449088-AE1A-4C38-833D-4403073AC979}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
   </bookViews>
   <sheets>
-    <sheet name="Worksheet" sheetId="1" r:id="rId1"/>
+    <sheet name="Worksheet" sheetId="1" r:id="rId4"/>
+    <sheet name="Info Kategori &amp; Rak" sheetId="2" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <definedNames/>
+  <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="81">
   <si>
     <t>kode_buku</t>
   </si>
@@ -52,39 +48,230 @@
     <t>stok_tersedia</t>
   </si>
   <si>
-    <t>kategori_id</t>
-  </si>
-  <si>
-    <t>rak_id</t>
+    <t>kode_kategori</t>
+  </si>
+  <si>
+    <t>kode_rak</t>
   </si>
   <si>
     <t>status</t>
   </si>
   <si>
-    <t>bku001</t>
-  </si>
-  <si>
-    <t>wuwung</t>
-  </si>
-  <si>
-    <t>ef</t>
-  </si>
-  <si>
-    <t>d</t>
-  </si>
-  <si>
-    <t>ffwf</t>
+    <t>B001</t>
+  </si>
+  <si>
+    <t>978-123-456-7890</t>
+  </si>
+  <si>
+    <t>Contoh Judul Buku</t>
+  </si>
+  <si>
+    <t>Nama Pengarang</t>
+  </si>
+  <si>
+    <t>Nama Penerbit</t>
+  </si>
+  <si>
+    <t>Deskripsi buku contoh</t>
+  </si>
+  <si>
+    <t>R600</t>
   </si>
   <si>
     <t>tersedia</t>
+  </si>
+  <si>
+    <t>INFORMASI KATEGORI DAN RAK</t>
+  </si>
+  <si>
+    <t>Gunakan KODE di bawah ini untuk mengisi kode_kategori dan kode_rak</t>
+  </si>
+  <si>
+    <t>KATEGORI:</t>
+  </si>
+  <si>
+    <t>Kode Kategori</t>
+  </si>
+  <si>
+    <t>Nama Kategori</t>
+  </si>
+  <si>
+    <t>Deskripsi</t>
+  </si>
+  <si>
+    <t>000</t>
+  </si>
+  <si>
+    <t>Komputer, Informasi dan Referensi umum</t>
+  </si>
+  <si>
+    <t>Buku-buku tentang komputer, informasi, dan referensi umum</t>
+  </si>
+  <si>
+    <t>Filsafat dan Psikologi</t>
+  </si>
+  <si>
+    <t>Buku-buku tentang filsafat dan psikologi</t>
+  </si>
+  <si>
+    <t>Agama</t>
+  </si>
+  <si>
+    <t>Buku-buku tentang agama</t>
+  </si>
+  <si>
+    <t>Ilmu Sosial</t>
+  </si>
+  <si>
+    <t>Buku-buku tentang ilmu sosial</t>
+  </si>
+  <si>
+    <t>Bahasa</t>
+  </si>
+  <si>
+    <t>Buku-buku tentang bahasa</t>
+  </si>
+  <si>
+    <t>Sains dan Matematika</t>
+  </si>
+  <si>
+    <t>Buku-buku tentang sains dan matematika</t>
+  </si>
+  <si>
+    <t>Teknologi</t>
+  </si>
+  <si>
+    <t>Buku-buku tentang teknologi</t>
+  </si>
+  <si>
+    <t>Kesenian dan Rekreasi</t>
+  </si>
+  <si>
+    <t>Buku-buku tentang kesenian dan rekreasi</t>
+  </si>
+  <si>
+    <t>Sastra</t>
+  </si>
+  <si>
+    <t>Buku-buku tentang sastra</t>
+  </si>
+  <si>
+    <t>Sejarah dan Geografi</t>
+  </si>
+  <si>
+    <t>Buku-buku tentang sejarah dan geografi</t>
+  </si>
+  <si>
+    <t>RAK:</t>
+  </si>
+  <si>
+    <t>Kode Rak</t>
+  </si>
+  <si>
+    <t>Nama Rak</t>
+  </si>
+  <si>
+    <t>Lokasi</t>
+  </si>
+  <si>
+    <t>R000</t>
+  </si>
+  <si>
+    <t>Rak Komputer &amp; Referensi</t>
+  </si>
+  <si>
+    <t>Rak 1 - Depan</t>
+  </si>
+  <si>
+    <t>R100</t>
+  </si>
+  <si>
+    <t>Rak Filsafat &amp; Psikologi</t>
+  </si>
+  <si>
+    <t>Rak 1 - Belakang</t>
+  </si>
+  <si>
+    <t>R200</t>
+  </si>
+  <si>
+    <t>Rak Agama</t>
+  </si>
+  <si>
+    <t>Rak 2 - Depan</t>
+  </si>
+  <si>
+    <t>R300</t>
+  </si>
+  <si>
+    <t>Rak Ilmu Sosial</t>
+  </si>
+  <si>
+    <t>Rak 2 - Belakang</t>
+  </si>
+  <si>
+    <t>R400</t>
+  </si>
+  <si>
+    <t>Rak Bahasa</t>
+  </si>
+  <si>
+    <t>Rak 3 - Depan</t>
+  </si>
+  <si>
+    <t>R500</t>
+  </si>
+  <si>
+    <t>Rak Sains &amp; Matematika</t>
+  </si>
+  <si>
+    <t>Rak 3 - Belakang</t>
+  </si>
+  <si>
+    <t>Rak Teknologi</t>
+  </si>
+  <si>
+    <t>Rak 4 - Depan</t>
+  </si>
+  <si>
+    <t>R700</t>
+  </si>
+  <si>
+    <t>Rak Seni &amp; Rekreasi</t>
+  </si>
+  <si>
+    <t>Rak 4 - Belakang</t>
+  </si>
+  <si>
+    <t>R800</t>
+  </si>
+  <si>
+    <t>Rak Sastra</t>
+  </si>
+  <si>
+    <t>Rak 5 - Depan</t>
+  </si>
+  <si>
+    <t>R900</t>
+  </si>
+  <si>
+    <t>Rak Sejarah &amp; Geografi</t>
+  </si>
+  <si>
+    <t>Rak 5 - Belakang</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -111,21 +298,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <tableStyles defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotTableStyle1"/>
 </styleSheet>
 </file>
 
@@ -415,11 +594,29 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xml:space="preserve" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
   <dimension ref="A1:M2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col min="1" max="1" width="11.711" bestFit="true" customWidth="true" style="0"/>
+    <col min="2" max="2" width="19.995" bestFit="true" customWidth="true" style="0"/>
+    <col min="3" max="3" width="21.138" bestFit="true" customWidth="true" style="0"/>
+    <col min="4" max="4" width="17.567" bestFit="true" customWidth="true" style="0"/>
+    <col min="5" max="5" width="16.425" bestFit="true" customWidth="true" style="0"/>
+    <col min="6" max="6" width="15.282" bestFit="true" customWidth="true" style="0"/>
+    <col min="7" max="7" width="17.567" bestFit="true" customWidth="true" style="0"/>
+    <col min="8" max="8" width="25.851" bestFit="true" customWidth="true" style="0"/>
+    <col min="9" max="9" width="12.854" bestFit="true" customWidth="true" style="0"/>
+    <col min="10" max="10" width="16.425" bestFit="true" customWidth="true" style="0"/>
+    <col min="11" max="11" width="16.425" bestFit="true" customWidth="true" style="0"/>
+    <col min="12" max="12" width="10.569" bestFit="true" customWidth="true" style="0"/>
+    <col min="13" max="13" width="10.569" bestFit="true" customWidth="true" style="0"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -460,48 +657,303 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13">
       <c r="A2" t="s">
         <v>13</v>
       </c>
-      <c r="B2">
-        <v>123</v>
+      <c r="B2" t="s">
+        <v>14</v>
       </c>
       <c r="C2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F2">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="G2">
-        <v>2</v>
+        <v>200</v>
       </c>
       <c r="H2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I2">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K2">
-        <v>1</v>
-      </c>
-      <c r="L2">
-        <v>1</v>
+        <v>600</v>
+      </c>
+      <c r="L2" t="s">
+        <v>19</v>
       </c>
       <c r="M2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
+  <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xml:space="preserve" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
+  <dimension ref="A1:G15"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" spans="1:7">
+      <c r="A1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E5" t="s">
+        <v>49</v>
+      </c>
+      <c r="F5" t="s">
+        <v>50</v>
+      </c>
+      <c r="G5" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" t="s">
+        <v>29</v>
+      </c>
+      <c r="E6" t="s">
+        <v>52</v>
+      </c>
+      <c r="F6" t="s">
+        <v>53</v>
+      </c>
+      <c r="G6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7">
+        <v>100</v>
+      </c>
+      <c r="B7" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" t="s">
+        <v>31</v>
+      </c>
+      <c r="E7" t="s">
+        <v>55</v>
+      </c>
+      <c r="F7" t="s">
+        <v>56</v>
+      </c>
+      <c r="G7" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8">
+        <v>200</v>
+      </c>
+      <c r="B8" t="s">
+        <v>32</v>
+      </c>
+      <c r="C8" t="s">
+        <v>33</v>
+      </c>
+      <c r="E8" t="s">
+        <v>58</v>
+      </c>
+      <c r="F8" t="s">
+        <v>59</v>
+      </c>
+      <c r="G8" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9">
+        <v>300</v>
+      </c>
+      <c r="B9" t="s">
+        <v>34</v>
+      </c>
+      <c r="C9" t="s">
+        <v>35</v>
+      </c>
+      <c r="E9" t="s">
+        <v>61</v>
+      </c>
+      <c r="F9" t="s">
+        <v>62</v>
+      </c>
+      <c r="G9" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10">
+        <v>400</v>
+      </c>
+      <c r="B10" t="s">
+        <v>36</v>
+      </c>
+      <c r="C10" t="s">
+        <v>37</v>
+      </c>
+      <c r="E10" t="s">
+        <v>64</v>
+      </c>
+      <c r="F10" t="s">
+        <v>65</v>
+      </c>
+      <c r="G10" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11">
+        <v>500</v>
+      </c>
+      <c r="B11" t="s">
+        <v>38</v>
+      </c>
+      <c r="C11" t="s">
+        <v>39</v>
+      </c>
+      <c r="E11" t="s">
+        <v>67</v>
+      </c>
+      <c r="F11" t="s">
+        <v>68</v>
+      </c>
+      <c r="G11" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12">
+        <v>600</v>
+      </c>
+      <c r="B12" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12" t="s">
+        <v>41</v>
+      </c>
+      <c r="E12" t="s">
+        <v>19</v>
+      </c>
+      <c r="F12" t="s">
+        <v>70</v>
+      </c>
+      <c r="G12" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13">
+        <v>700</v>
+      </c>
+      <c r="B13" t="s">
+        <v>42</v>
+      </c>
+      <c r="C13" t="s">
+        <v>43</v>
+      </c>
+      <c r="E13" t="s">
+        <v>72</v>
+      </c>
+      <c r="F13" t="s">
+        <v>73</v>
+      </c>
+      <c r="G13" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14">
+        <v>800</v>
+      </c>
+      <c r="B14" t="s">
+        <v>44</v>
+      </c>
+      <c r="C14" t="s">
+        <v>45</v>
+      </c>
+      <c r="E14" t="s">
+        <v>75</v>
+      </c>
+      <c r="F14" t="s">
+        <v>76</v>
+      </c>
+      <c r="G14" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="A15">
+        <v>900</v>
+      </c>
+      <c r="B15" t="s">
+        <v>46</v>
+      </c>
+      <c r="C15" t="s">
+        <v>47</v>
+      </c>
+      <c r="E15" t="s">
+        <v>78</v>
+      </c>
+      <c r="F15" t="s">
+        <v>79</v>
+      </c>
+      <c r="G15" t="s">
+        <v>80</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions gridLines="false" gridLinesSet="true"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
 </worksheet>
 </file>
</xml_diff>